<commit_message>
making edit to allow for double single peaks
</commit_message>
<xml_diff>
--- a/BeatnotePostCombFix/Apr06,2026/April6_NewFits.xlsx
+++ b/BeatnotePostCombFix/Apr06,2026/April6_NewFits.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wolfwalker\Documents\git\6s7p\BeatnotePostCombFix\Apr06,2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostCombFix\Apr06,2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5EC5AE9-CF73-43D7-BEF2-45A151F5C34F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAAE0EAB-8882-4CA5-8D74-8117189E0568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{DE27D4D9-8A5E-4A81-9645-FB782B2C9508}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE27D4D9-8A5E-4A81-9645-FB782B2C9508}"/>
   </bookViews>
   <sheets>
     <sheet name="456" sheetId="1" r:id="rId1"/>
@@ -30,12 +30,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="28">
   <si>
     <t>Date</t>
   </si>
@@ -125,7 +128,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -140,8 +143,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -151,6 +168,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -163,11 +190,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -175,9 +204,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Good" xfId="2" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -487,7 +525,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -495,6 +532,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -530,356 +568,6 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>PwrWings</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="38100" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'456'!$H$2:$H$17</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
-                <c:pt idx="0">
-                  <c:v>6.5217247454024503E-3</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>5.9524002287284303E-3</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>5.7833937165545097E-3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>5.6772585844044104E-3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>5.2723851850779201E-3</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5.7736330999529802E-3</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>5.4820542543049999E-3</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>5.3264612042161E-3</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>7.7412677657778999E-3</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>7.62516583333779E-3</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>7.3898611584532698E-3</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>5.4621766338067397E-3</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>7.8243799858341203E-3</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>5.3787315766305899E-3</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>7.5747441774043902E-3</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>7.6964905441190001E-3</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4877-4E33-965D-6C04C86DE9A3}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="1093716624"/>
-        <c:axId val="1093719952"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="1093716624"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1093719952"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="1093719952"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1093716624"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1159,7 +847,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1167,6 +854,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1201,7 +889,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1481,7 +1169,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1489,6 +1176,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1643,46 +1331,6 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -3231,536 +2879,20 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>368300</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>28574</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>577850</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>161924</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>445485</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>78936</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>83535</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>31311</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3785,42 +2917,6 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>776287</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>576262</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DEA20ED6-8683-4714-8506-509498556F15}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3829,15 +2925,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>111125</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>225425</xdr:rowOff>
+      <xdr:colOff>330200</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>349250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>447675</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>22225</xdr:rowOff>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>327025</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4219,15 +3315,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E67E67-BE51-40B6-BF6A-AB076C1A076C}">
   <dimension ref="A1:X19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="17.6328125" customWidth="1"/>
-    <col min="10" max="10" width="16.453125" customWidth="1"/>
-    <col min="16" max="16" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.625" customWidth="1"/>
+    <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.5" customWidth="1"/>
+    <col min="16" max="16" width="12.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:24">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4253,7 +3355,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:24">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -4300,7 +3402,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:24">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -4329,35 +3431,35 @@
         <v>23</v>
       </c>
       <c r="K3">
-        <f>AVERAGE(B2:B19)</f>
+        <f t="shared" ref="K3:Q3" si="0">AVERAGE(B2:B19)</f>
         <v>0.18223766556713897</v>
       </c>
       <c r="L3">
-        <f>AVERAGE(C2:C19)</f>
+        <f t="shared" si="0"/>
         <v>1.3311203169335977</v>
       </c>
       <c r="M3">
-        <f>AVERAGE(D2:D19)</f>
+        <f t="shared" si="0"/>
         <v>-1.3598659716220023E-3</v>
       </c>
       <c r="N3">
-        <f>AVERAGE(E2:E19)</f>
+        <f t="shared" si="0"/>
         <v>2.4215668828125128</v>
       </c>
       <c r="O3">
-        <f>AVERAGE(F2:F19)</f>
+        <f t="shared" si="0"/>
         <v>41.813359767150573</v>
       </c>
       <c r="P3">
-        <f>AVERAGE(G2:G19)</f>
+        <f t="shared" si="0"/>
         <v>7.5215001461198126E-4</v>
       </c>
       <c r="Q3">
-        <f>AVERAGE(H2:H19)</f>
+        <f t="shared" si="0"/>
         <v>6.4051330433753505E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:24">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -4414,7 +3516,7 @@
         <v>1.0350004003727045E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:24">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -4443,35 +3545,35 @@
         <v>25</v>
       </c>
       <c r="K5">
-        <f t="shared" ref="K5:Q5" si="0">K4/K3*100</f>
+        <f t="shared" ref="K5:Q5" si="1">K4/K3*100</f>
         <v>1.3109842428238778</v>
       </c>
       <c r="L5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.13541189170358062</v>
       </c>
       <c r="M5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-17.795680208612989</v>
       </c>
       <c r="N5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>28.015244965395837</v>
       </c>
       <c r="O5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4.1420674102852137</v>
       </c>
       <c r="P5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.9774889770268235E-14</v>
       </c>
       <c r="Q5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>16.15892118655016</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:24">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -4504,83 +3606,105 @@
         <v>0.32774606070596946</v>
       </c>
       <c r="L6">
-        <f t="shared" ref="L6:Q6" si="1">L5/SQRT(16)</f>
+        <f t="shared" ref="L6:Q6" si="2">L5/SQRT(16)</f>
         <v>3.3852972925895154E-2</v>
       </c>
       <c r="M6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-4.4489200521532473</v>
       </c>
       <c r="N6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.0038112413489593</v>
       </c>
       <c r="O6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.0355168525713034</v>
       </c>
       <c r="P6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.4437224425670588E-15</v>
       </c>
       <c r="Q6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.0397302966375399</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:24">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="2">
         <v>0.18120694450344099</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="2">
         <v>1.3314337765094799</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="2">
         <v>-7.1625116325157502E-4</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>3.3523854443785299</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="2">
         <v>40.4387541848401</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7" s="2">
         <v>7.5215001461198105E-4</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>5.7736330999529802E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:24">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="2">
         <v>0.18339176159659801</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="2">
         <v>1.33218831237308</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>-1.37990713885699E-3</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>2.4004485807738298</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="2">
         <v>40.379300673643698</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="2">
         <v>7.5215001461198105E-4</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>5.4820542543049999E-3</v>
       </c>
+      <c r="J8" s="4"/>
+      <c r="K8" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:24">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -4605,8 +3729,39 @@
       <c r="H9" s="1">
         <v>5.3264612042161E-3</v>
       </c>
+      <c r="J9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K9" s="4">
+        <f>AVERAGE(B2:B6,B9:B15)</f>
+        <v>0.18223123464258348</v>
+      </c>
+      <c r="L9" s="4">
+        <f t="shared" ref="L9:Q9" si="3">AVERAGE(C2:C6,C9:C15)</f>
+        <v>1.3315736860131067</v>
+      </c>
+      <c r="M9" s="4">
+        <f t="shared" si="3"/>
+        <v>-1.4244675461433968E-3</v>
+      </c>
+      <c r="N9" s="4">
+        <f t="shared" si="3"/>
+        <v>2.3897641086739023</v>
+      </c>
+      <c r="O9" s="4">
+        <f t="shared" si="3"/>
+        <v>41.816801047398563</v>
+      </c>
+      <c r="P9" s="4">
+        <f t="shared" si="3"/>
+        <v>7.5215001461198105E-4</v>
+      </c>
+      <c r="Q9" s="4">
+        <f t="shared" si="3"/>
+        <v>6.3296005515186861E-3</v>
+      </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:24">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -4631,8 +3786,39 @@
       <c r="H10" s="1">
         <v>7.7412677657778999E-3</v>
       </c>
+      <c r="J10" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="4">
+        <f>_xlfn.STDEV.S(B2:B6,B9:B15)</f>
+        <v>2.455751422895953E-3</v>
+      </c>
+      <c r="L10" s="4">
+        <f t="shared" ref="L10:Q10" si="4">_xlfn.STDEV.S(C2:C6,C9:C15)</f>
+        <v>1.4064247882405341E-3</v>
+      </c>
+      <c r="M10" s="4">
+        <f t="shared" si="4"/>
+        <v>1.902305921248247E-4</v>
+      </c>
+      <c r="N10" s="4">
+        <f t="shared" si="4"/>
+        <v>0.69967355315699598</v>
+      </c>
+      <c r="O10" s="4">
+        <f t="shared" si="4"/>
+        <v>1.7875948689722638</v>
+      </c>
+      <c r="P10" s="4">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4">
+        <f t="shared" si="4"/>
+        <v>1.0319207384430055E-3</v>
+      </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:24">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -4657,8 +3843,39 @@
       <c r="H11" s="1">
         <v>7.62516583333779E-3</v>
       </c>
+      <c r="J11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K11" s="4">
+        <f>K10/K9*100</f>
+        <v>1.3476018135488708</v>
+      </c>
+      <c r="L11" s="4">
+        <f t="shared" ref="K11:Q11" si="5">L10/L9*100</f>
+        <v>0.10562125123180684</v>
+      </c>
+      <c r="M11" s="4">
+        <f t="shared" si="5"/>
+        <v>-13.35450517211536</v>
+      </c>
+      <c r="N11" s="4">
+        <f t="shared" si="5"/>
+        <v>29.27793377670443</v>
+      </c>
+      <c r="O11" s="4">
+        <f t="shared" si="5"/>
+        <v>4.2748245303270771</v>
+      </c>
+      <c r="P11" s="4">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4">
+        <f t="shared" si="5"/>
+        <v>16.303094169116449</v>
+      </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:24">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -4683,8 +3900,39 @@
       <c r="H12" s="1">
         <v>7.3898611584532698E-3</v>
       </c>
+      <c r="J12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K12" s="4">
+        <f>K11/SQRT(16)</f>
+        <v>0.33690045338721769</v>
+      </c>
+      <c r="L12" s="4">
+        <f t="shared" ref="L12:Q12" si="6">L11/SQRT(16)</f>
+        <v>2.6405312807951709E-2</v>
+      </c>
+      <c r="M12" s="4">
+        <f t="shared" si="6"/>
+        <v>-3.33862629302884</v>
+      </c>
+      <c r="N12" s="4">
+        <f t="shared" si="6"/>
+        <v>7.3194834441761074</v>
+      </c>
+      <c r="O12" s="4">
+        <f t="shared" si="6"/>
+        <v>1.0687061325817693</v>
+      </c>
+      <c r="P12" s="4">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4">
+        <f t="shared" si="6"/>
+        <v>4.0757735422791121</v>
+      </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:24">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -4710,7 +3958,7 @@
         <v>5.4621766338067397E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:24">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -4736,7 +3984,7 @@
         <v>7.8243799858341203E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:24">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -4766,59 +4014,59 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:24">
+      <c r="A16" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="3">
         <v>0.17930907427498799</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="3">
         <v>1.32774141310028</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="3">
         <v>-1.2384555806072999E-3</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="3">
         <v>1.65745758544111</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16" s="3">
         <v>42.1801149943445</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G16" s="3">
         <v>7.5215001461198105E-4</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="3">
         <v>7.5747441774043902E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:8">
+      <c r="A17" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="2">
         <v>0.18512005298819501</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="2">
         <v>1.3276773367974399</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>-1.3296311095154099E-3</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>2.6576092103199098</v>
       </c>
-      <c r="F17" s="1">
+      <c r="F17" s="2">
         <v>44.213973852798098</v>
       </c>
-      <c r="G17" s="1">
+      <c r="G17" s="2">
         <v>7.5215001461198105E-4</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>7.6964905441190001E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -4828,7 +4076,7 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -4847,19 +4095,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6499FFC7-3DA5-4057-863B-C101A2BD7DDC}">
   <dimension ref="A1:Q16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" customWidth="1"/>
-    <col min="2" max="3" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.75" customWidth="1"/>
+    <col min="2" max="3" width="11.375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
-    <col min="16" max="16" width="15.7265625" customWidth="1"/>
+    <col min="16" max="16" width="15.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4885,7 +4133,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" ht="42.75">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -4932,7 +4180,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" ht="42.75">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -4965,31 +4213,31 @@
         <v>9.5834711291571395</v>
       </c>
       <c r="L3">
-        <f>AVERAGE(C2:C8,C9:C15)</f>
+        <f t="shared" ref="L3:Q3" si="0">AVERAGE(C2:C8,C9:C15)</f>
         <v>1.162153889491518</v>
       </c>
       <c r="M3">
-        <f>AVERAGE(D2:D8,D9:D15)</f>
+        <f t="shared" si="0"/>
         <v>-1.5025398128554247E-3</v>
       </c>
       <c r="N3">
-        <f>AVERAGE(E2:E8,E9:E15)</f>
+        <f t="shared" si="0"/>
         <v>2.6608399668835325</v>
       </c>
       <c r="O3">
-        <f>AVERAGE(F2:F8,F9:F15)</f>
+        <f t="shared" si="0"/>
         <v>42.320636854563752</v>
       </c>
       <c r="P3">
-        <f>AVERAGE(G2:G8,G9:G15)</f>
+        <f t="shared" si="0"/>
         <v>2.2873004957013996E-3</v>
       </c>
       <c r="Q3">
-        <f>AVERAGE(H2:H8,H9:H15)</f>
+        <f t="shared" si="0"/>
         <v>3.9599068935265838E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" ht="42.75">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -5022,31 +4270,31 @@
         <v>9.7066723913118894E-2</v>
       </c>
       <c r="L4">
-        <f>_xlfn.STDEV.S(C2:C8,C9:C15)</f>
+        <f t="shared" ref="L4:Q4" si="1">_xlfn.STDEV.S(C2:C8,C9:C15)</f>
         <v>5.3432058427090486E-3</v>
       </c>
       <c r="M4">
-        <f>_xlfn.STDEV.S(D2:D8,D9:D15)</f>
+        <f t="shared" si="1"/>
         <v>8.83693924068583E-4</v>
       </c>
       <c r="N4">
-        <f>_xlfn.STDEV.S(E2:E8,E9:E15)</f>
+        <f t="shared" si="1"/>
         <v>0.47761963009070002</v>
       </c>
       <c r="O4">
-        <f>_xlfn.STDEV.S(F2:F8,F9:F15)</f>
+        <f t="shared" si="1"/>
         <v>0.99692067221831782</v>
       </c>
       <c r="P4">
-        <f>_xlfn.STDEV.S(G2:G8,G9:G15)</f>
+        <f t="shared" si="1"/>
         <v>4.5005190690732244E-19</v>
       </c>
       <c r="Q4">
-        <f>_xlfn.STDEV.S(H2:H8,H9:H15)</f>
+        <f t="shared" si="1"/>
         <v>8.4798007481810031E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" ht="42.75">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -5072,7 +4320,7 @@
         <v>3.88277049890592E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" ht="42.75">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -5113,23 +4361,23 @@
         <v>-58.813345011418519</v>
       </c>
       <c r="N6">
-        <f t="shared" ref="N6:Q6" si="0">N4/N3*100</f>
+        <f t="shared" ref="N6:Q6" si="2">N4/N3*100</f>
         <v>17.949957007377058</v>
       </c>
       <c r="O6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.3556372170018807</v>
       </c>
       <c r="P6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.9676116354327736E-14</v>
       </c>
       <c r="Q6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2.1414141736623322</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" ht="42.75">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
@@ -5154,12 +4402,8 @@
       <c r="H7" s="2">
         <v>3.8909036436339001E-2</v>
       </c>
-      <c r="K7">
-        <f>K6/SQRT(18)</f>
-        <v>0.23873235414569227</v>
-      </c>
     </row>
-    <row r="8" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" ht="42.75">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -5184,36 +4428,30 @@
       <c r="H8" s="2">
         <v>3.8407947485241803E-2</v>
       </c>
-      <c r="K8">
-        <f>(B7-K3)/K3</f>
-        <v>-1.7607868580085138E-2</v>
-      </c>
-      <c r="L8">
-        <f>(C7-L3)/L3</f>
-        <v>5.0027107926781519E-3</v>
-      </c>
-      <c r="M8">
-        <f>(D7-M3)/M3</f>
-        <v>1.8945188972388154</v>
-      </c>
-      <c r="N8">
-        <f>(E7-N3)/N3</f>
-        <v>-0.30024366804968439</v>
-      </c>
-      <c r="O8">
-        <f>(F7-O3)/O3</f>
-        <v>8.0787930557046014E-3</v>
-      </c>
-      <c r="P8">
-        <f>(G7-P3)/P3</f>
-        <v>1.8960380142846676E-16</v>
-      </c>
-      <c r="Q8">
-        <f>(H7-Q3)/Q3</f>
-        <v>-1.7425472807324354E-2</v>
+      <c r="J8" s="4"/>
+      <c r="K8" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" ht="42.75">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -5238,36 +4476,39 @@
       <c r="H9" s="1">
         <v>4.0124607725458297E-2</v>
       </c>
-      <c r="K9">
-        <f>(B8-K3)/K3</f>
-        <v>-1.8806952601880634E-2</v>
-      </c>
-      <c r="L9">
-        <f>(C8-L3)/L3</f>
-        <v>3.2274908401528713E-3</v>
-      </c>
-      <c r="M9">
-        <f>(D8-M3)/M3</f>
-        <v>-9.775845698181726E-2</v>
-      </c>
-      <c r="N9">
-        <f>(E8-N3)/N3</f>
-        <v>0.14326178507179757</v>
-      </c>
-      <c r="O9">
-        <f>(F8-O3)/O3</f>
-        <v>4.2328082793673033E-2</v>
-      </c>
-      <c r="P9">
-        <f>(G8-P3)/P3</f>
-        <v>1.8960380142846676E-16</v>
-      </c>
-      <c r="Q9">
-        <f>(H8-Q3)/Q3</f>
-        <v>-3.0079531717556503E-2</v>
+      <c r="J9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K9" s="4">
+        <f>AVERAGE(B2:B6,B9:B15)</f>
+        <v>9.6265982288147658</v>
+      </c>
+      <c r="L9" s="4">
+        <f>AVERAGE(C2:C6,C9:C15)</f>
+        <v>1.1613568260882767</v>
+      </c>
+      <c r="M9" s="4">
+        <f t="shared" ref="L9:Q9" si="3">AVERAGE(D2:D6,D9:D15)</f>
+        <v>-1.2775644715512762E-3</v>
+      </c>
+      <c r="N9" s="4">
+        <f t="shared" si="3"/>
+        <v>2.6956486059088824</v>
+      </c>
+      <c r="O9" s="4">
+        <f t="shared" si="3"/>
+        <v>42.142865930580861</v>
+      </c>
+      <c r="P9" s="4">
+        <f t="shared" si="3"/>
+        <v>2.2873004957013996E-3</v>
+      </c>
+      <c r="Q9" s="4">
+        <f t="shared" si="3"/>
+        <v>3.9755831764345086E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" ht="42.75">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -5292,8 +4533,39 @@
       <c r="H10" s="1">
         <v>4.0161020680797598E-2</v>
       </c>
+      <c r="J10" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="4">
+        <f>_xlfn.STDEV.S(B2:B6,B9:B15)</f>
+        <v>4.2874966127329557E-2</v>
+      </c>
+      <c r="L10" s="4">
+        <f t="shared" ref="L10:Q10" si="4">_xlfn.STDEV.S(C2:C6,C9:C15)</f>
+        <v>5.3568464265952532E-3</v>
+      </c>
+      <c r="M10" s="4">
+        <f t="shared" si="4"/>
+        <v>3.5927667312676337E-4</v>
+      </c>
+      <c r="N10" s="4">
+        <f t="shared" si="4"/>
+        <v>0.44389538733979811</v>
+      </c>
+      <c r="O10" s="4">
+        <f t="shared" si="4"/>
+        <v>0.91527419813041777</v>
+      </c>
+      <c r="P10" s="4">
+        <f t="shared" si="4"/>
+        <v>4.5296489464404432E-19</v>
+      </c>
+      <c r="Q10" s="4">
+        <f t="shared" si="4"/>
+        <v>8.0668246098657451E-4</v>
+      </c>
     </row>
-    <row r="11" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" ht="42.75">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -5318,8 +4590,39 @@
       <c r="H11" s="1">
         <v>4.01957931520791E-2</v>
       </c>
+      <c r="J11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K11" s="4">
+        <f>K10/K9*100</f>
+        <v>0.4453802382548207</v>
+      </c>
+      <c r="L11" s="4">
+        <f>L10/L9*100</f>
+        <v>0.46125758304950709</v>
+      </c>
+      <c r="M11" s="4">
+        <f>M10/M9*100</f>
+        <v>-28.1219994080231</v>
+      </c>
+      <c r="N11" s="4">
+        <f>N10/N9*100</f>
+        <v>16.46710874580522</v>
+      </c>
+      <c r="O11" s="4">
+        <f>O10/O9*100</f>
+        <v>2.1718366274331888</v>
+      </c>
+      <c r="P11" s="4">
+        <f>P10/P9*100</f>
+        <v>1.9803471187774254E-14</v>
+      </c>
+      <c r="Q11" s="4">
+        <f>Q10/Q9*100</f>
+        <v>2.0290921487147595</v>
+      </c>
     </row>
-    <row r="12" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" ht="42.75">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -5344,36 +4647,8 @@
       <c r="H12" s="1">
         <v>4.0627807408899798E-2</v>
       </c>
-      <c r="K12">
-        <f>AVERAGE(B2:B6,B9:B15)</f>
-        <v>9.6265982288147658</v>
-      </c>
-      <c r="L12">
-        <f t="shared" ref="L12:Q12" si="1">AVERAGE(C2:C6,C9:C15)</f>
-        <v>1.1613568260882767</v>
-      </c>
-      <c r="M12">
-        <f t="shared" si="1"/>
-        <v>-1.2775644715512762E-3</v>
-      </c>
-      <c r="N12">
-        <f t="shared" si="1"/>
-        <v>2.6956486059088824</v>
-      </c>
-      <c r="O12">
-        <f t="shared" si="1"/>
-        <v>42.142865930580861</v>
-      </c>
-      <c r="P12">
-        <f t="shared" si="1"/>
-        <v>2.2873004957013996E-3</v>
-      </c>
-      <c r="Q12">
-        <f t="shared" si="1"/>
-        <v>3.9755831764345086E-2</v>
-      </c>
     </row>
-    <row r="13" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" ht="42.75">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -5398,36 +4673,8 @@
       <c r="H13" s="1">
         <v>3.9807036376995002E-2</v>
       </c>
-      <c r="K13">
-        <f>_xlfn.STDEV.S(B2:B6,B18:B25)</f>
-        <v>5.4049589437203442E-2</v>
-      </c>
-      <c r="L13">
-        <f t="shared" ref="L13:Q13" si="2">_xlfn.STDEV.S(C2:C6,C18:C25)</f>
-        <v>8.8165250409120489E-4</v>
-      </c>
-      <c r="M13">
-        <f t="shared" si="2"/>
-        <v>2.2594438519616905E-4</v>
-      </c>
-      <c r="N13">
-        <f t="shared" si="2"/>
-        <v>7.6919691136686607E-4</v>
-      </c>
-      <c r="O13">
-        <f t="shared" si="2"/>
-        <v>0.91457320606724857</v>
-      </c>
-      <c r="P13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q13">
-        <f t="shared" si="2"/>
-        <v>1.0200284707886839E-3</v>
-      </c>
     </row>
-    <row r="14" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" ht="42.75">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -5452,12 +4699,8 @@
       <c r="H14" s="1">
         <v>3.9800928551067302E-2</v>
       </c>
-      <c r="K14">
-        <f>K13/K12*100</f>
-        <v>0.56146094552299675</v>
-      </c>
     </row>
-    <row r="15" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" ht="42.75">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -5482,12 +4725,8 @@
       <c r="H15" s="1">
         <v>4.0279009963469802E-2</v>
       </c>
-      <c r="K15">
-        <f>K14/COUNT(B2:B6,B9:B15)</f>
-        <v>4.6788412126916396E-2</v>
-      </c>
     </row>
-    <row r="16" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" ht="42.75">
       <c r="A16" s="2" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
neeed to fix 894 residuals
</commit_message>
<xml_diff>
--- a/BeatnotePostCombFix/Apr06,2026/April6_NewFits.xlsx
+++ b/BeatnotePostCombFix/Apr06,2026/April6_NewFits.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostCombFix\Apr06,2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wolfwalker\Documents\git\6s7p\BeatnotePostCombFix\Apr06,2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAAE0EAB-8882-4CA5-8D74-8117189E0568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63BDDF2B-2F4F-4EDF-B7C7-29C945AA1F5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE27D4D9-8A5E-4A81-9645-FB782B2C9508}"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{DE27D4D9-8A5E-4A81-9645-FB782B2C9508}"/>
   </bookViews>
   <sheets>
     <sheet name="456" sheetId="1" r:id="rId1"/>
@@ -29,9 +29,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -128,7 +125,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -525,6 +522,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -532,7 +530,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -847,6 +844,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -854,7 +852,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1169,6 +1166,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1176,7 +1174,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2883,16 +2880,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>577850</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>161924</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>180974</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>83535</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>31311</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>96235</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>50361</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3315,21 +3312,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E67E67-BE51-40B6-BF6A-AB076C1A076C}">
   <dimension ref="A1:X19"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="17.625" customWidth="1"/>
-    <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.5" customWidth="1"/>
-    <col min="16" max="16" width="12.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6328125" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.453125" customWidth="1"/>
+    <col min="16" max="16" width="12.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3355,7 +3352,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -3402,7 +3399,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3459,7 +3456,7 @@
         <v>6.4051330433753505E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -3516,7 +3513,7 @@
         <v>1.0350004003727045E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -3545,11 +3542,11 @@
         <v>25</v>
       </c>
       <c r="K5">
-        <f t="shared" ref="K5:Q5" si="1">K4/K3*100</f>
+        <f>K4/K3*100</f>
         <v>1.3109842428238778</v>
       </c>
       <c r="L5">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="K5:Q5" si="1">L4/L3*100</f>
         <v>0.13541189170358062</v>
       </c>
       <c r="M5">
@@ -3573,7 +3570,7 @@
         <v>16.15892118655016</v>
       </c>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -3602,8 +3599,8 @@
         <v>27</v>
       </c>
       <c r="K6">
-        <f>K5/SQRT(16)</f>
-        <v>0.32774606070596946</v>
+        <f>K5/COUNT(B2:B17)</f>
+        <v>8.1936515176492364E-2</v>
       </c>
       <c r="L6">
         <f t="shared" ref="L6:Q6" si="2">L5/SQRT(16)</f>
@@ -3630,7 +3627,7 @@
         <v>4.0397302966375399</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
@@ -3656,7 +3653,7 @@
         <v>5.7736330999529802E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -3704,7 +3701,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -3761,7 +3758,7 @@
         <v>6.3296005515186861E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -3818,7 +3815,7 @@
         <v>1.0319207384430055E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -3851,7 +3848,7 @@
         <v>1.3476018135488708</v>
       </c>
       <c r="L11" s="4">
-        <f t="shared" ref="K11:Q11" si="5">L10/L9*100</f>
+        <f t="shared" ref="L11:Q11" si="5">L10/L9*100</f>
         <v>0.10562125123180684</v>
       </c>
       <c r="M11" s="4">
@@ -3875,7 +3872,7 @@
         <v>16.303094169116449</v>
       </c>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -3932,7 +3929,7 @@
         <v>4.0757735422791121</v>
       </c>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -3958,7 +3955,7 @@
         <v>5.4621766338067397E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -3984,7 +3981,7 @@
         <v>7.8243799858341203E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -4014,7 +4011,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>22</v>
       </c>
@@ -4040,7 +4037,7 @@
         <v>7.5747441774043902E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>26</v>
       </c>
@@ -4066,7 +4063,7 @@
         <v>7.6964905441190001E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -4076,7 +4073,7 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -4095,19 +4092,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6499FFC7-3DA5-4057-863B-C101A2BD7DDC}">
   <dimension ref="A1:Q16"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.75" customWidth="1"/>
-    <col min="2" max="3" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7265625" customWidth="1"/>
+    <col min="2" max="3" width="11.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.36328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
-    <col min="16" max="16" width="15.75" customWidth="1"/>
+    <col min="16" max="16" width="15.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4133,7 +4130,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="42.75">
+    <row r="2" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -4180,7 +4177,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="42.75">
+    <row r="3" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -4237,7 +4234,7 @@
         <v>3.9599068935265838E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="42.75">
+    <row r="4" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -4294,7 +4291,7 @@
         <v>8.4798007481810031E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="42.75">
+    <row r="5" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -4320,7 +4317,7 @@
         <v>3.88277049890592E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="42.75">
+    <row r="6" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -4377,7 +4374,7 @@
         <v>2.1414141736623322</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="42.75">
+    <row r="7" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
@@ -4403,7 +4400,7 @@
         <v>3.8909036436339001E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="42.75">
+    <row r="8" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -4451,7 +4448,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="42.75">
+    <row r="9" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -4488,7 +4485,7 @@
         <v>1.1613568260882767</v>
       </c>
       <c r="M9" s="4">
-        <f t="shared" ref="L9:Q9" si="3">AVERAGE(D2:D6,D9:D15)</f>
+        <f t="shared" ref="M9:Q9" si="3">AVERAGE(D2:D6,D9:D15)</f>
         <v>-1.2775644715512762E-3</v>
       </c>
       <c r="N9" s="4">
@@ -4508,7 +4505,7 @@
         <v>3.9755831764345086E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="42.75">
+    <row r="10" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -4565,7 +4562,7 @@
         <v>8.0668246098657451E-4</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="42.75">
+    <row r="11" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -4598,31 +4595,31 @@
         <v>0.4453802382548207</v>
       </c>
       <c r="L11" s="4">
-        <f>L10/L9*100</f>
+        <f t="shared" ref="K11:Q11" si="5">L10/L9*100</f>
         <v>0.46125758304950709</v>
       </c>
       <c r="M11" s="4">
-        <f>M10/M9*100</f>
+        <f t="shared" si="5"/>
         <v>-28.1219994080231</v>
       </c>
       <c r="N11" s="4">
-        <f>N10/N9*100</f>
+        <f t="shared" si="5"/>
         <v>16.46710874580522</v>
       </c>
       <c r="O11" s="4">
-        <f>O10/O9*100</f>
+        <f t="shared" si="5"/>
         <v>2.1718366274331888</v>
       </c>
       <c r="P11" s="4">
-        <f>P10/P9*100</f>
+        <f t="shared" si="5"/>
         <v>1.9803471187774254E-14</v>
       </c>
       <c r="Q11" s="4">
-        <f>Q10/Q9*100</f>
+        <f t="shared" si="5"/>
         <v>2.0290921487147595</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="42.75">
+    <row r="12" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -4648,7 +4645,7 @@
         <v>4.0627807408899798E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="42.75">
+    <row r="13" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -4674,7 +4671,7 @@
         <v>3.9807036376995002E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="42.75">
+    <row r="14" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -4700,7 +4697,7 @@
         <v>3.9800928551067302E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="42.75">
+    <row r="15" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -4726,7 +4723,7 @@
         <v>4.0279009963469802E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="42.75">
+    <row r="16" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>26</v>
       </c>

</xml_diff>